<commit_message>
daily order build 2026-09-13
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-14
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-15
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-16
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-17
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-18
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>92017</v>
+        <v>88555</v>
       </c>
       <c r="D2" t="n">
-        <v>47319</v>
+        <v>46527</v>
       </c>
       <c r="E2" t="n">
-        <v>27749</v>
+        <v>24963</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>502</v>
+        <v>467</v>
       </c>
       <c r="C3" t="n">
-        <v>438511</v>
+        <v>404595</v>
       </c>
       <c r="D3" t="n">
-        <v>199403</v>
+        <v>195161</v>
       </c>
       <c r="E3" t="n">
-        <v>211799</v>
+        <v>183532</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C4" t="n">
-        <v>135339</v>
+        <v>129534</v>
       </c>
       <c r="D4" t="n">
-        <v>64774</v>
+        <v>64142</v>
       </c>
       <c r="E4" t="n">
-        <v>140146</v>
+        <v>137204</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C5" t="n">
-        <v>295717</v>
+        <v>273144</v>
       </c>
       <c r="D5" t="n">
-        <v>112280</v>
+        <v>103468</v>
       </c>
       <c r="E5" t="n">
-        <v>228787</v>
+        <v>215615</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C6" t="n">
-        <v>28562</v>
+        <v>26971</v>
       </c>
       <c r="D6" t="n">
-        <v>16342</v>
+        <v>14510</v>
       </c>
       <c r="E6" t="n">
-        <v>8558</v>
+        <v>8960</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-19
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C2" t="n">
-        <v>88555</v>
+        <v>92634</v>
       </c>
       <c r="D2" t="n">
-        <v>46527</v>
+        <v>48472</v>
       </c>
       <c r="E2" t="n">
-        <v>24963</v>
+        <v>27651</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>467</v>
+        <v>520</v>
       </c>
       <c r="C3" t="n">
-        <v>404595</v>
+        <v>448236</v>
       </c>
       <c r="D3" t="n">
-        <v>195161</v>
+        <v>202545</v>
       </c>
       <c r="E3" t="n">
-        <v>183532</v>
+        <v>220054</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="C4" t="n">
-        <v>129534</v>
+        <v>140712</v>
       </c>
       <c r="D4" t="n">
-        <v>64142</v>
+        <v>69625</v>
       </c>
       <c r="E4" t="n">
-        <v>137204</v>
+        <v>147201</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="C5" t="n">
-        <v>273144</v>
+        <v>302284</v>
       </c>
       <c r="D5" t="n">
-        <v>103468</v>
+        <v>111122</v>
       </c>
       <c r="E5" t="n">
-        <v>215615</v>
+        <v>237077</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>26971</v>
+        <v>22882</v>
       </c>
       <c r="D6" t="n">
-        <v>14510</v>
+        <v>12387</v>
       </c>
       <c r="E6" t="n">
-        <v>8960</v>
+        <v>7043</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-20
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C2" t="n">
-        <v>92634</v>
+        <v>98967</v>
       </c>
       <c r="D2" t="n">
-        <v>48472</v>
+        <v>51050</v>
       </c>
       <c r="E2" t="n">
-        <v>27651</v>
+        <v>31485</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>520</v>
+        <v>571</v>
       </c>
       <c r="C3" t="n">
-        <v>448236</v>
+        <v>493340</v>
       </c>
       <c r="D3" t="n">
-        <v>202545</v>
+        <v>209419</v>
       </c>
       <c r="E3" t="n">
-        <v>220054</v>
+        <v>258693</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="C4" t="n">
-        <v>140712</v>
+        <v>151287</v>
       </c>
       <c r="D4" t="n">
-        <v>69625</v>
+        <v>75785</v>
       </c>
       <c r="E4" t="n">
-        <v>147201</v>
+        <v>153956</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="C5" t="n">
-        <v>302284</v>
+        <v>334666</v>
       </c>
       <c r="D5" t="n">
-        <v>111122</v>
+        <v>122998</v>
       </c>
       <c r="E5" t="n">
-        <v>237077</v>
+        <v>249031</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C6" t="n">
-        <v>22882</v>
+        <v>25637</v>
       </c>
       <c r="D6" t="n">
-        <v>12387</v>
+        <v>13608</v>
       </c>
       <c r="E6" t="n">
-        <v>7043</v>
+        <v>8274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-21
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="C2" t="n">
-        <v>98967</v>
+        <v>90682</v>
       </c>
       <c r="D2" t="n">
-        <v>51050</v>
+        <v>45899</v>
       </c>
       <c r="E2" t="n">
-        <v>31485</v>
+        <v>27435</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>571</v>
+        <v>542</v>
       </c>
       <c r="C3" t="n">
-        <v>493340</v>
+        <v>437550</v>
       </c>
       <c r="D3" t="n">
-        <v>209419</v>
+        <v>201013</v>
       </c>
       <c r="E3" t="n">
-        <v>258693</v>
+        <v>210573</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C4" t="n">
-        <v>151287</v>
+        <v>155801</v>
       </c>
       <c r="D4" t="n">
-        <v>75785</v>
+        <v>73555</v>
       </c>
       <c r="E4" t="n">
-        <v>153956</v>
+        <v>164569</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="C5" t="n">
-        <v>334666</v>
+        <v>320459</v>
       </c>
       <c r="D5" t="n">
-        <v>122998</v>
+        <v>120644</v>
       </c>
       <c r="E5" t="n">
-        <v>249031</v>
+        <v>236855</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>25637</v>
+        <v>24358</v>
       </c>
       <c r="D6" t="n">
-        <v>13608</v>
+        <v>13062</v>
       </c>
       <c r="E6" t="n">
-        <v>8274</v>
+        <v>7664</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-22
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C2" t="n">
-        <v>90682</v>
+        <v>93003</v>
       </c>
       <c r="D2" t="n">
-        <v>45899</v>
+        <v>47063</v>
       </c>
       <c r="E2" t="n">
-        <v>27435</v>
+        <v>28444</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>542</v>
+        <v>531</v>
       </c>
       <c r="C3" t="n">
-        <v>437550</v>
+        <v>428899</v>
       </c>
       <c r="D3" t="n">
-        <v>201013</v>
+        <v>199885</v>
       </c>
       <c r="E3" t="n">
-        <v>210573</v>
+        <v>203085</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         <v>189</v>
       </c>
       <c r="C4" t="n">
-        <v>155801</v>
+        <v>158490</v>
       </c>
       <c r="D4" t="n">
-        <v>73555</v>
+        <v>74897</v>
       </c>
       <c r="E4" t="n">
-        <v>164569</v>
+        <v>165494</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C5" t="n">
-        <v>320459</v>
+        <v>321143</v>
       </c>
       <c r="D5" t="n">
-        <v>120644</v>
+        <v>122277</v>
       </c>
       <c r="E5" t="n">
-        <v>236855</v>
+        <v>233410</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C6" t="n">
-        <v>24358</v>
+        <v>23547</v>
       </c>
       <c r="D6" t="n">
-        <v>13062</v>
+        <v>13120</v>
       </c>
       <c r="E6" t="n">
-        <v>7664</v>
+        <v>6982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-23
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C2" t="n">
         <v>96757</v>
@@ -459,7 +459,7 @@
         <v>49553</v>
       </c>
       <c r="E2" t="n">
-        <v>30302</v>
+        <v>30438</v>
       </c>
     </row>
     <row r="3">
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="C3" t="n">
         <v>431221</v>
@@ -478,7 +478,7 @@
         <v>196805</v>
       </c>
       <c r="E3" t="n">
-        <v>208540</v>
+        <v>209593</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
daily order build 2026-09-24
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-25
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-26
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C2" t="n">
-        <v>89667</v>
+        <v>94200</v>
       </c>
       <c r="D2" t="n">
-        <v>46002</v>
+        <v>47483</v>
       </c>
       <c r="E2" t="n">
-        <v>27550</v>
+        <v>30566</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>485</v>
+        <v>534</v>
       </c>
       <c r="C3" t="n">
-        <v>396865</v>
+        <v>434070</v>
       </c>
       <c r="D3" t="n">
-        <v>197127</v>
+        <v>207818</v>
       </c>
       <c r="E3" t="n">
-        <v>172758</v>
+        <v>199474</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="C4" t="n">
-        <v>140220</v>
+        <v>156678</v>
       </c>
       <c r="D4" t="n">
-        <v>69408</v>
+        <v>74125</v>
       </c>
       <c r="E4" t="n">
-        <v>115209</v>
+        <v>128454</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>170</v>
+        <v>195</v>
       </c>
       <c r="C5" t="n">
-        <v>262434</v>
+        <v>309876</v>
       </c>
       <c r="D5" t="n">
-        <v>109600</v>
+        <v>123124</v>
       </c>
       <c r="E5" t="n">
-        <v>214106</v>
+        <v>241744</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
-        <v>23107</v>
+        <v>23323</v>
       </c>
       <c r="D6" t="n">
-        <v>12084</v>
+        <v>12720</v>
       </c>
       <c r="E6" t="n">
-        <v>7607</v>
+        <v>7291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-27
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C2" t="n">
-        <v>94200</v>
+        <v>102341</v>
       </c>
       <c r="D2" t="n">
-        <v>47483</v>
+        <v>51134</v>
       </c>
       <c r="E2" t="n">
-        <v>30566</v>
+        <v>33996</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>534</v>
+        <v>588</v>
       </c>
       <c r="C3" t="n">
-        <v>434070</v>
+        <v>478111</v>
       </c>
       <c r="D3" t="n">
-        <v>207818</v>
+        <v>213617</v>
       </c>
       <c r="E3" t="n">
-        <v>199474</v>
+        <v>238939</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C4" t="n">
-        <v>156678</v>
+        <v>166383</v>
       </c>
       <c r="D4" t="n">
-        <v>74125</v>
+        <v>77646</v>
       </c>
       <c r="E4" t="n">
-        <v>128454</v>
+        <v>135320</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="C5" t="n">
-        <v>309876</v>
+        <v>346645</v>
       </c>
       <c r="D5" t="n">
-        <v>123124</v>
+        <v>130519</v>
       </c>
       <c r="E5" t="n">
-        <v>241744</v>
+        <v>264286</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C6" t="n">
-        <v>23323</v>
+        <v>25165</v>
       </c>
       <c r="D6" t="n">
-        <v>12720</v>
+        <v>13375</v>
       </c>
       <c r="E6" t="n">
-        <v>7291</v>
+        <v>8425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-09-29
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-09-30
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-01
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C2" t="n">
-        <v>99671</v>
+        <v>95888</v>
       </c>
       <c r="D2" t="n">
-        <v>50367</v>
+        <v>52565</v>
       </c>
       <c r="E2" t="n">
-        <v>32710</v>
+        <v>26325</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>561</v>
+        <v>534</v>
       </c>
       <c r="C3" t="n">
-        <v>427054</v>
+        <v>422288</v>
       </c>
       <c r="D3" t="n">
-        <v>204769</v>
+        <v>205475</v>
       </c>
       <c r="E3" t="n">
-        <v>204835</v>
+        <v>198410</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="C4" t="n">
-        <v>168042</v>
+        <v>129461</v>
       </c>
       <c r="D4" t="n">
-        <v>77750</v>
+        <v>68069</v>
       </c>
       <c r="E4" t="n">
-        <v>135837</v>
+        <v>69550</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>206</v>
+        <v>156</v>
       </c>
       <c r="C5" t="n">
-        <v>352022</v>
+        <v>278074</v>
       </c>
       <c r="D5" t="n">
-        <v>132394</v>
+        <v>125253</v>
       </c>
       <c r="E5" t="n">
-        <v>252815</v>
+        <v>141696</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C6" t="n">
-        <v>22703</v>
+        <v>20338</v>
       </c>
       <c r="D6" t="n">
-        <v>11683</v>
+        <v>10491</v>
       </c>
       <c r="E6" t="n">
-        <v>7593</v>
+        <v>6751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-02
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C2" t="n">
-        <v>95888</v>
+        <v>93920</v>
       </c>
       <c r="D2" t="n">
-        <v>52565</v>
+        <v>50690</v>
       </c>
       <c r="E2" t="n">
-        <v>26325</v>
+        <v>25570</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>534</v>
+        <v>493</v>
       </c>
       <c r="C3" t="n">
-        <v>422288</v>
+        <v>390534</v>
       </c>
       <c r="D3" t="n">
-        <v>205475</v>
+        <v>191770</v>
       </c>
       <c r="E3" t="n">
-        <v>198410</v>
+        <v>180838</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="C4" t="n">
-        <v>129461</v>
+        <v>107144</v>
       </c>
       <c r="D4" t="n">
-        <v>68069</v>
+        <v>60200</v>
       </c>
       <c r="E4" t="n">
-        <v>69550</v>
+        <v>63810</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C5" t="n">
-        <v>278074</v>
+        <v>235548</v>
       </c>
       <c r="D5" t="n">
-        <v>125253</v>
+        <v>102730</v>
       </c>
       <c r="E5" t="n">
-        <v>141696</v>
+        <v>133841</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C6" t="n">
-        <v>20338</v>
+        <v>18706</v>
       </c>
       <c r="D6" t="n">
-        <v>10491</v>
+        <v>9555</v>
       </c>
       <c r="E6" t="n">
-        <v>6751</v>
+        <v>6156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-03
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-04
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C2" t="n">
-        <v>100597</v>
+        <v>107037</v>
       </c>
       <c r="D2" t="n">
-        <v>55181</v>
+        <v>57284</v>
       </c>
       <c r="E2" t="n">
-        <v>26621</v>
+        <v>30883</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>520</v>
+        <v>563</v>
       </c>
       <c r="C3" t="n">
-        <v>429997</v>
+        <v>464633</v>
       </c>
       <c r="D3" t="n">
-        <v>207091</v>
+        <v>211882</v>
       </c>
       <c r="E3" t="n">
-        <v>196114</v>
+        <v>226932</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="C4" t="n">
-        <v>121826</v>
+        <v>128611</v>
       </c>
       <c r="D4" t="n">
-        <v>67067</v>
+        <v>69755</v>
       </c>
       <c r="E4" t="n">
-        <v>65666</v>
+        <v>68563</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C5" t="n">
-        <v>275478</v>
+        <v>302046</v>
       </c>
       <c r="D5" t="n">
-        <v>113247</v>
+        <v>118405</v>
       </c>
       <c r="E5" t="n">
-        <v>148945</v>
+        <v>156854</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C6" t="n">
-        <v>19498</v>
+        <v>21726</v>
       </c>
       <c r="D6" t="n">
-        <v>10324</v>
+        <v>11323</v>
       </c>
       <c r="E6" t="n">
-        <v>6287</v>
+        <v>7410</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-06
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C2" t="n">
-        <v>107037</v>
+        <v>100762</v>
       </c>
       <c r="D2" t="n">
-        <v>57284</v>
+        <v>54442</v>
       </c>
       <c r="E2" t="n">
-        <v>30883</v>
+        <v>27557</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>563</v>
+        <v>507</v>
       </c>
       <c r="C3" t="n">
-        <v>464633</v>
+        <v>418416</v>
       </c>
       <c r="D3" t="n">
-        <v>211882</v>
+        <v>202574</v>
       </c>
       <c r="E3" t="n">
-        <v>226831</v>
+        <v>189799</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C4" t="n">
-        <v>128611</v>
+        <v>132759</v>
       </c>
       <c r="D4" t="n">
-        <v>69755</v>
+        <v>69607</v>
       </c>
       <c r="E4" t="n">
-        <v>68367</v>
+        <v>71254</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C5" t="n">
-        <v>302046</v>
+        <v>295305</v>
       </c>
       <c r="D5" t="n">
-        <v>118405</v>
+        <v>115476</v>
       </c>
       <c r="E5" t="n">
-        <v>157175</v>
+        <v>152356</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C6" t="n">
-        <v>21726</v>
+        <v>20739</v>
       </c>
       <c r="D6" t="n">
-        <v>11323</v>
+        <v>11010</v>
       </c>
       <c r="E6" t="n">
-        <v>7410</v>
+        <v>6768</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-08
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -453,13 +453,13 @@
         <v>81</v>
       </c>
       <c r="C2" t="n">
-        <v>98862</v>
+        <v>99035</v>
       </c>
       <c r="D2" t="n">
-        <v>52218</v>
+        <v>52030</v>
       </c>
       <c r="E2" t="n">
-        <v>27956</v>
+        <v>28638</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="C3" t="n">
-        <v>403803</v>
+        <v>401133</v>
       </c>
       <c r="D3" t="n">
-        <v>197684</v>
+        <v>198424</v>
       </c>
       <c r="E3" t="n">
-        <v>180696</v>
+        <v>176893</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C4" t="n">
-        <v>134205</v>
+        <v>139932</v>
       </c>
       <c r="D4" t="n">
-        <v>68908</v>
+        <v>69475</v>
       </c>
       <c r="E4" t="n">
-        <v>71947</v>
+        <v>76690</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C5" t="n">
-        <v>293233</v>
+        <v>303594</v>
       </c>
       <c r="D5" t="n">
-        <v>114986</v>
+        <v>116608</v>
       </c>
       <c r="E5" t="n">
-        <v>151741</v>
+        <v>154311</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" t="n">
-        <v>20285</v>
+        <v>20305</v>
       </c>
       <c r="D6" t="n">
-        <v>11084</v>
+        <v>10864</v>
       </c>
       <c r="E6" t="n">
-        <v>6223</v>
+        <v>6412</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-09
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-10
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-11
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C2" t="n">
-        <v>94877</v>
+        <v>102888</v>
       </c>
       <c r="D2" t="n">
-        <v>48019</v>
+        <v>50096</v>
       </c>
       <c r="E2" t="n">
-        <v>30443</v>
+        <v>34862</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>515</v>
+        <v>567</v>
       </c>
       <c r="C3" t="n">
-        <v>399269</v>
+        <v>444251</v>
       </c>
       <c r="D3" t="n">
-        <v>190143</v>
+        <v>195643</v>
       </c>
       <c r="E3" t="n">
-        <v>183869</v>
+        <v>222512</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C4" t="n">
-        <v>133579</v>
+        <v>142607</v>
       </c>
       <c r="D4" t="n">
-        <v>61459</v>
+        <v>64918</v>
       </c>
       <c r="E4" t="n">
-        <v>85392</v>
+        <v>89386</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="C5" t="n">
-        <v>272253</v>
+        <v>306825</v>
       </c>
       <c r="D5" t="n">
-        <v>107902</v>
+        <v>115741</v>
       </c>
       <c r="E5" t="n">
-        <v>154596</v>
+        <v>171771</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C6" t="n">
-        <v>23495</v>
+        <v>25620</v>
       </c>
       <c r="D6" t="n">
-        <v>12646</v>
+        <v>13353</v>
       </c>
       <c r="E6" t="n">
-        <v>8125</v>
+        <v>9357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-13
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C2" t="n">
-        <v>102888</v>
+        <v>99243</v>
       </c>
       <c r="D2" t="n">
-        <v>50096</v>
+        <v>48245</v>
       </c>
       <c r="E2" t="n">
-        <v>34862</v>
+        <v>33441</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>567</v>
+        <v>523</v>
       </c>
       <c r="C3" t="n">
-        <v>444251</v>
+        <v>385952</v>
       </c>
       <c r="D3" t="n">
-        <v>195643</v>
+        <v>185993</v>
       </c>
       <c r="E3" t="n">
-        <v>222512</v>
+        <v>174414</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C4" t="n">
-        <v>142607</v>
+        <v>141237</v>
       </c>
       <c r="D4" t="n">
-        <v>64918</v>
+        <v>63341</v>
       </c>
       <c r="E4" t="n">
-        <v>89386</v>
+        <v>88286</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C5" t="n">
-        <v>306825</v>
+        <v>284327</v>
       </c>
       <c r="D5" t="n">
-        <v>115741</v>
+        <v>107635</v>
       </c>
       <c r="E5" t="n">
-        <v>171771</v>
+        <v>159065</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C6" t="n">
-        <v>25620</v>
+        <v>24542</v>
       </c>
       <c r="D6" t="n">
-        <v>13353</v>
+        <v>12666</v>
       </c>
       <c r="E6" t="n">
-        <v>9357</v>
+        <v>8832</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-14
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-15
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C2" t="n">
-        <v>101626</v>
+        <v>97359</v>
       </c>
       <c r="D2" t="n">
-        <v>46540</v>
+        <v>45492</v>
       </c>
       <c r="E2" t="n">
-        <v>37068</v>
+        <v>34658</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>507</v>
+        <v>484</v>
       </c>
       <c r="C3" t="n">
-        <v>377324</v>
+        <v>359464</v>
       </c>
       <c r="D3" t="n">
-        <v>180026</v>
+        <v>174849</v>
       </c>
       <c r="E3" t="n">
-        <v>170441</v>
+        <v>158435</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C4" t="n">
-        <v>148612</v>
+        <v>139283</v>
       </c>
       <c r="D4" t="n">
-        <v>65262</v>
+        <v>61195</v>
       </c>
       <c r="E4" t="n">
-        <v>92545</v>
+        <v>88608</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="C5" t="n">
-        <v>305221</v>
+        <v>266248</v>
       </c>
       <c r="D5" t="n">
-        <v>114125</v>
+        <v>107299</v>
       </c>
       <c r="E5" t="n">
-        <v>165445</v>
+        <v>140111</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C6" t="n">
-        <v>24486</v>
+        <v>22440</v>
       </c>
       <c r="D6" t="n">
-        <v>12857</v>
+        <v>12256</v>
       </c>
       <c r="E6" t="n">
-        <v>8411</v>
+        <v>6787</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-16
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C2" t="n">
-        <v>97359</v>
+        <v>99182</v>
       </c>
       <c r="D2" t="n">
-        <v>45492</v>
+        <v>45717</v>
       </c>
       <c r="E2" t="n">
-        <v>34658</v>
+        <v>36023</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>484</v>
+        <v>469</v>
       </c>
       <c r="C3" t="n">
-        <v>359464</v>
+        <v>348732</v>
       </c>
       <c r="D3" t="n">
-        <v>174849</v>
+        <v>172433</v>
       </c>
       <c r="E3" t="n">
-        <v>158435</v>
+        <v>150484</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C4" t="n">
-        <v>139283</v>
+        <v>137335</v>
       </c>
       <c r="D4" t="n">
-        <v>61195</v>
+        <v>61623</v>
       </c>
       <c r="E4" t="n">
-        <v>88608</v>
+        <v>82505</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="C5" t="n">
-        <v>266248</v>
+        <v>258607</v>
       </c>
       <c r="D5" t="n">
-        <v>107299</v>
+        <v>102334</v>
       </c>
       <c r="E5" t="n">
-        <v>140111</v>
+        <v>138643</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C6" t="n">
-        <v>22440</v>
+        <v>20500</v>
       </c>
       <c r="D6" t="n">
-        <v>12256</v>
+        <v>11589</v>
       </c>
       <c r="E6" t="n">
-        <v>6787</v>
+        <v>5832</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-17
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="C2" t="n">
-        <v>99182</v>
+        <v>115333</v>
       </c>
       <c r="D2" t="n">
-        <v>45717</v>
+        <v>49670</v>
       </c>
       <c r="E2" t="n">
-        <v>36023</v>
+        <v>47753</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>469</v>
+        <v>530</v>
       </c>
       <c r="C3" t="n">
-        <v>348732</v>
+        <v>401323</v>
       </c>
       <c r="D3" t="n">
-        <v>172433</v>
+        <v>180168</v>
       </c>
       <c r="E3" t="n">
-        <v>150484</v>
+        <v>195680</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C4" t="n">
-        <v>137335</v>
+        <v>151482</v>
       </c>
       <c r="D4" t="n">
-        <v>61623</v>
+        <v>68342</v>
       </c>
       <c r="E4" t="n">
-        <v>82505</v>
+        <v>90731</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="C5" t="n">
-        <v>258607</v>
+        <v>300269</v>
       </c>
       <c r="D5" t="n">
-        <v>102334</v>
+        <v>114756</v>
       </c>
       <c r="E5" t="n">
-        <v>138643</v>
+        <v>159723</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C6" t="n">
-        <v>20500</v>
+        <v>21696</v>
       </c>
       <c r="D6" t="n">
-        <v>11589</v>
+        <v>12029</v>
       </c>
       <c r="E6" t="n">
-        <v>5832</v>
+        <v>6784</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-18
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>115333</v>
+        <v>123419</v>
       </c>
       <c r="D2" t="n">
-        <v>49670</v>
+        <v>50931</v>
       </c>
       <c r="E2" t="n">
-        <v>47753</v>
+        <v>53396</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>530</v>
+        <v>571</v>
       </c>
       <c r="C3" t="n">
-        <v>401323</v>
+        <v>435871</v>
       </c>
       <c r="D3" t="n">
-        <v>180168</v>
+        <v>184810</v>
       </c>
       <c r="E3" t="n">
-        <v>195680</v>
+        <v>226387</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C4" t="n">
-        <v>151482</v>
+        <v>160208</v>
       </c>
       <c r="D4" t="n">
-        <v>68342</v>
+        <v>70032</v>
       </c>
       <c r="E4" t="n">
-        <v>90731</v>
+        <v>99104</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="C5" t="n">
-        <v>300269</v>
+        <v>330642</v>
       </c>
       <c r="D5" t="n">
-        <v>114756</v>
+        <v>123446</v>
       </c>
       <c r="E5" t="n">
-        <v>159723</v>
+        <v>173725</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C6" t="n">
-        <v>21696</v>
+        <v>23157</v>
       </c>
       <c r="D6" t="n">
-        <v>12029</v>
+        <v>12840</v>
       </c>
       <c r="E6" t="n">
-        <v>6784</v>
+        <v>7357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-19
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C2" t="n">
-        <v>123419</v>
+        <v>112663</v>
       </c>
       <c r="D2" t="n">
-        <v>50931</v>
+        <v>48731</v>
       </c>
       <c r="E2" t="n">
-        <v>53396</v>
+        <v>45743</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>571</v>
+        <v>492</v>
       </c>
       <c r="C3" t="n">
-        <v>435871</v>
+        <v>367611</v>
       </c>
       <c r="D3" t="n">
-        <v>184810</v>
+        <v>176518</v>
       </c>
       <c r="E3" t="n">
-        <v>226387</v>
+        <v>166835</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C4" t="n">
-        <v>160208</v>
+        <v>159597</v>
       </c>
       <c r="D4" t="n">
-        <v>70032</v>
+        <v>69752</v>
       </c>
       <c r="E4" t="n">
-        <v>99104</v>
+        <v>98317</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C5" t="n">
-        <v>330642</v>
+        <v>315875</v>
       </c>
       <c r="D5" t="n">
-        <v>123446</v>
+        <v>118639</v>
       </c>
       <c r="E5" t="n">
-        <v>173725</v>
+        <v>166377</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" t="n">
-        <v>23157</v>
+        <v>21981</v>
       </c>
       <c r="D6" t="n">
-        <v>12840</v>
+        <v>12253</v>
       </c>
       <c r="E6" t="n">
-        <v>7357</v>
+        <v>7086</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-20
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C2" t="n">
-        <v>112663</v>
+        <v>110555</v>
       </c>
       <c r="D2" t="n">
-        <v>48731</v>
+        <v>44159</v>
       </c>
       <c r="E2" t="n">
-        <v>45743</v>
+        <v>47604</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>492</v>
+        <v>472</v>
       </c>
       <c r="C3" t="n">
-        <v>367611</v>
+        <v>357076</v>
       </c>
       <c r="D3" t="n">
-        <v>176518</v>
+        <v>175310</v>
       </c>
       <c r="E3" t="n">
-        <v>166835</v>
+        <v>157149</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C4" t="n">
-        <v>159597</v>
+        <v>160800</v>
       </c>
       <c r="D4" t="n">
-        <v>69752</v>
+        <v>68546</v>
       </c>
       <c r="E4" t="n">
-        <v>98317</v>
+        <v>106545</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="C5" t="n">
-        <v>315875</v>
+        <v>313200</v>
       </c>
       <c r="D5" t="n">
-        <v>118639</v>
+        <v>118418</v>
       </c>
       <c r="E5" t="n">
-        <v>166377</v>
+        <v>160824</v>
       </c>
     </row>
     <row r="6">
@@ -529,13 +529,13 @@
         <v>59</v>
       </c>
       <c r="C6" t="n">
-        <v>21981</v>
+        <v>21337</v>
       </c>
       <c r="D6" t="n">
-        <v>12253</v>
+        <v>11833</v>
       </c>
       <c r="E6" t="n">
-        <v>7086</v>
+        <v>6692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-21
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-22
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C2" t="n">
-        <v>114016</v>
+        <v>104055</v>
       </c>
       <c r="D2" t="n">
-        <v>46427</v>
+        <v>45985</v>
       </c>
       <c r="E2" t="n">
-        <v>48817</v>
+        <v>39283</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>471</v>
+        <v>462</v>
       </c>
       <c r="C3" t="n">
-        <v>358098</v>
+        <v>355121</v>
       </c>
       <c r="D3" t="n">
-        <v>175101</v>
+        <v>178907</v>
       </c>
       <c r="E3" t="n">
-        <v>158950</v>
+        <v>152088</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="C4" t="n">
-        <v>164388</v>
+        <v>132562</v>
       </c>
       <c r="D4" t="n">
-        <v>70152</v>
+        <v>62264</v>
       </c>
       <c r="E4" t="n">
-        <v>101042</v>
+        <v>80216</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>171</v>
+        <v>142</v>
       </c>
       <c r="C5" t="n">
-        <v>329627</v>
+        <v>251818</v>
       </c>
       <c r="D5" t="n">
-        <v>122403</v>
+        <v>105731</v>
       </c>
       <c r="E5" t="n">
-        <v>173749</v>
+        <v>139160</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C6" t="n">
-        <v>21694</v>
+        <v>22124</v>
       </c>
       <c r="D6" t="n">
-        <v>11995</v>
+        <v>12196</v>
       </c>
       <c r="E6" t="n">
-        <v>6808</v>
+        <v>7145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-23
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-24
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-25
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="C2" t="n">
-        <v>114113</v>
+        <v>124133</v>
       </c>
       <c r="D2" t="n">
-        <v>47588</v>
+        <v>49366</v>
       </c>
       <c r="E2" t="n">
-        <v>45598</v>
+        <v>53341</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>485</v>
+        <v>562</v>
       </c>
       <c r="C3" t="n">
-        <v>377263</v>
+        <v>445456</v>
       </c>
       <c r="D3" t="n">
-        <v>176122</v>
+        <v>183330</v>
       </c>
       <c r="E3" t="n">
-        <v>175440</v>
+        <v>237907</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C4" t="n">
-        <v>134320</v>
+        <v>146064</v>
       </c>
       <c r="D4" t="n">
-        <v>61521</v>
+        <v>64531</v>
       </c>
       <c r="E4" t="n">
-        <v>81137</v>
+        <v>93758</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="C5" t="n">
-        <v>276710</v>
+        <v>329495</v>
       </c>
       <c r="D5" t="n">
-        <v>112190</v>
+        <v>126815</v>
       </c>
       <c r="E5" t="n">
-        <v>156258</v>
+        <v>178344</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="C6" t="n">
-        <v>19735</v>
+        <v>23195</v>
       </c>
       <c r="D6" t="n">
-        <v>10917</v>
+        <v>12172</v>
       </c>
       <c r="E6" t="n">
-        <v>6023</v>
+        <v>8238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-26
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="C2" t="n">
-        <v>124133</v>
+        <v>112606</v>
       </c>
       <c r="D2" t="n">
-        <v>49366</v>
+        <v>43731</v>
       </c>
       <c r="E2" t="n">
-        <v>53341</v>
+        <v>48442</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>562</v>
+        <v>523</v>
       </c>
       <c r="C3" t="n">
-        <v>445456</v>
+        <v>391992</v>
       </c>
       <c r="D3" t="n">
-        <v>183330</v>
+        <v>178361</v>
       </c>
       <c r="E3" t="n">
-        <v>237907</v>
+        <v>189160</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C4" t="n">
-        <v>146064</v>
+        <v>148121</v>
       </c>
       <c r="D4" t="n">
-        <v>64531</v>
+        <v>65781</v>
       </c>
       <c r="E4" t="n">
-        <v>93758</v>
+        <v>93543</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C5" t="n">
-        <v>329495</v>
+        <v>322412</v>
       </c>
       <c r="D5" t="n">
-        <v>126815</v>
+        <v>125683</v>
       </c>
       <c r="E5" t="n">
-        <v>178344</v>
+        <v>172599</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6" t="n">
-        <v>23195</v>
+        <v>21179</v>
       </c>
       <c r="D6" t="n">
-        <v>12172</v>
+        <v>10799</v>
       </c>
       <c r="E6" t="n">
-        <v>8238</v>
+        <v>7501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily order build 2026-10-27
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-29
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
daily order build 2026-10-30
</commit_message>
<xml_diff>
--- a/data/All Dept Order Summary.xlsx
+++ b/data/All Dept Order Summary.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C2" t="n">
-        <v>108105</v>
+        <v>108239</v>
       </c>
       <c r="D2" t="n">
-        <v>45471</v>
+        <v>43858</v>
       </c>
       <c r="E2" t="n">
-        <v>40686</v>
+        <v>42787</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>511</v>
+        <v>496</v>
       </c>
       <c r="C3" t="n">
-        <v>394168</v>
+        <v>387705</v>
       </c>
       <c r="D3" t="n">
-        <v>179128</v>
+        <v>184792</v>
       </c>
       <c r="E3" t="n">
-        <v>189845</v>
+        <v>178007</v>
       </c>
     </row>
     <row r="4">
@@ -488,16 +488,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="C4" t="n">
-        <v>127449</v>
+        <v>108200</v>
       </c>
       <c r="D4" t="n">
-        <v>59523</v>
+        <v>53778</v>
       </c>
       <c r="E4" t="n">
-        <v>74673</v>
+        <v>64782</v>
       </c>
     </row>
     <row r="5">
@@ -507,16 +507,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C5" t="n">
-        <v>294418</v>
+        <v>291723</v>
       </c>
       <c r="D5" t="n">
-        <v>120656</v>
+        <v>117652</v>
       </c>
       <c r="E5" t="n">
-        <v>161886</v>
+        <v>146634</v>
       </c>
     </row>
     <row r="6">
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C6" t="n">
-        <v>19703</v>
+        <v>21126</v>
       </c>
       <c r="D6" t="n">
-        <v>10847</v>
+        <v>11456</v>
       </c>
       <c r="E6" t="n">
-        <v>5716</v>
+        <v>6509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>